<commit_message>
chore: expand sample docs to 1800-37000 chars each (based on real Chinese regulations)
</commit_message>
<xml_diff>
--- a/data/docs/行政/采购分级标准.xlsx
+++ b/data/docs/行政/采购分级标准.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,63 +424,254 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>采购方式</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>比价要求</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>审批层级</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>是否需招标</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>招标方式</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>合同要求</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>付款条件</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>&lt;1000</t>
+          <t>500以下</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>直接采购</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>部门主管</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>否</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>货到付款</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1000-10000</t>
+          <t>500-1000</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>比价采购</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>至少2家</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>部门负责人</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>否</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>货到付款</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>&gt;10000</t>
+          <t>1000-5000</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>比价采购</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>至少3家</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>部门负责人</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>简易采购合同</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>验收后15日内</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5000-50000</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>询价采购</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>至少3家</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>部门负责人+财务总监</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>邀请招标</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>正式合同</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>验收后30日内</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>50000-200000</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>公开招标</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>至少5家</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>总经理</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>是</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>公开招标</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>正式合同+履约保函</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>预付30%，验收后付60%，质保期满付10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>20万以上</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>公开招标+专家评审</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>至少5家+外部专家</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>总经理+董事会备案</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>公开招标+外部专家评审</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>正式合同+履约保函+质量保证金</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>按合同分期</t>
         </is>
       </c>
     </row>

</xml_diff>